<commit_message>
Add AveriGo E2E suite (averigoE2E) and latest module suites
</commit_message>
<xml_diff>
--- a/micromarketservices/data/MicroMarketCreationPage.xlsx
+++ b/micromarketservices/data/MicroMarketCreationPage.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="35">
   <si>
     <t xml:space="preserve">Username</t>
   </si>
@@ -102,19 +102,22 @@
     <t xml:space="preserve">01/07/2025</t>
   </si>
   <si>
+    <t xml:space="preserve">Coke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Coke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GSG Market </t>
+  </si>
+  <si>
     <t xml:space="preserve">Milky Way</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Coke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GSG Market </t>
   </si>
   <si>
     <t xml:space="preserve">-10</t>
@@ -531,7 +534,7 @@
         <v>16</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>27</v>
@@ -579,7 +582,7 @@
         <v>16</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>27</v>
@@ -629,16 +632,16 @@
         <v>16</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P5" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -728,7 +731,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>19</v>
@@ -758,7 +761,7 @@
         <v>16</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>27</v>

</xml_diff>